<commit_message>
Fix export polish across all download formats
- PNG/PDF: плашка счётчика по ширине подписи + склонение (рекорд/рекорда/рекордов)
- PNG/PDF: составы эстафет переносятся на 1–2 строки (строка выше), обрезка
  с многоточием вместо канвас-сжатия, «(бассейн 25 м)» убран из дисциплины —
  бассейн уже в колонке «Категория»
- PDF: JPEG вместо PNG внутри (был 108 МБ несжатого растра — стало ~3 МБ)
- XLSX: Consolas вместо Menlo (есть на Windows), результаты моно и вправо,
  в т.ч. на сводном листе
- TXT: шапка с источником и датой, ширины колонок по данным —
  эстафеты больше не ломают сетку
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -35,7 +35,7 @@
       <color rgb="00FAFAFA"/>
     </font>
     <font>
-      <name val="Menlo"/>
+      <name val="Consolas"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,7 +68,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -523,12 +525,12 @@
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>27.23</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>27.23</t>
         </is>
@@ -571,12 +573,12 @@
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>27.23</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>27.23</t>
         </is>
@@ -619,12 +621,12 @@
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>29.52</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>29.52</t>
         </is>
@@ -667,12 +669,12 @@
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>25.30</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>25.30</t>
         </is>
@@ -715,12 +717,12 @@
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>24.20</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>24.20</t>
         </is>
@@ -763,12 +765,12 @@
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>58.18</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>58.18</t>
         </is>
@@ -811,12 +813,12 @@
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>1:04.36</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>64.36</t>
         </is>
@@ -859,12 +861,12 @@
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>56.42</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>56.42</t>
         </is>
@@ -907,12 +909,12 @@
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>52.98</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>52.98</t>
         </is>
@@ -955,12 +957,12 @@
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>2:04.94</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>124.94</t>
         </is>
@@ -1003,12 +1005,12 @@
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>2:17.55</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>137.55</t>
         </is>
@@ -1051,12 +1053,12 @@
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>2:07.33</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>127.33</t>
         </is>
@@ -1099,12 +1101,12 @@
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>1:55.08</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>115.08</t>
         </is>
@@ -1147,12 +1149,12 @@
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>2:09.56</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>129.56</t>
         </is>
@@ -1195,12 +1197,12 @@
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>4:04.10</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>244.10</t>
         </is>
@@ -1243,12 +1245,12 @@
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>4:36.25</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>276.25</t>
         </is>
@@ -1291,12 +1293,12 @@
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>8:18.77</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>498.77</t>
         </is>
@@ -1339,12 +1341,12 @@
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>15:50.22</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>950.22</t>
         </is>
@@ -1391,12 +1393,12 @@
           <t>Трофимова Дарья · Кузнецова Александра · Гайфутдинова Алина · Клепикова Дарья</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>3:34.69</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>214.69</t>
         </is>
@@ -1443,12 +1445,12 @@
           <t>Фесикова Анастасия · Ефимова Юлия · Чимрова Светлана · Попова Вероника</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>3:53.38</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>233.38</t>
         </is>
@@ -1495,12 +1497,12 @@
           <t>Егорова Анна · Гуженкова Анастасия · Саламатина Валерия · Андрусенко Вероника</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>7:48.25</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>468.25</t>
         </is>
@@ -1543,12 +1545,12 @@
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>25.60</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>25.60</t>
         </is>
@@ -1591,12 +1593,12 @@
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>29.08</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>29.08</t>
         </is>
@@ -1639,12 +1641,12 @@
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>24.58</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>24.58</t>
         </is>
@@ -1687,12 +1689,12 @@
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>23.34</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>23.34</t>
         </is>
@@ -1735,12 +1737,12 @@
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>55.83</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>55.83</t>
         </is>
@@ -1783,12 +1785,12 @@
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>1:02.91</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>62.91</t>
         </is>
@@ -1831,12 +1833,12 @@
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>55.63</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>55.63</t>
         </is>
@@ -1879,12 +1881,12 @@
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>51.62</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>51.62</t>
         </is>
@@ -1927,12 +1929,12 @@
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>57.59</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>57.59</t>
         </is>
@@ -1975,12 +1977,12 @@
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>2:01.57</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>121.57</t>
         </is>
@@ -2023,12 +2025,12 @@
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>2:14.70</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>134.70</t>
         </is>
@@ -2071,12 +2073,12 @@
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>2:03.76</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>123.76</t>
         </is>
@@ -2119,12 +2121,12 @@
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>1:52.46</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>112.46</t>
         </is>
@@ -2167,12 +2169,12 @@
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>2:06.79</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>126.79</t>
         </is>
@@ -2215,12 +2217,12 @@
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>3:58.25</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>238.25</t>
         </is>
@@ -2263,12 +2265,12 @@
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>4:31.13</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>271.13</t>
         </is>
@@ -2311,12 +2313,12 @@
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>8:04.65</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>484.65</t>
         </is>
@@ -2359,12 +2361,12 @@
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>15:18.30</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>918.30</t>
         </is>
@@ -2411,12 +2413,12 @@
           <t>Насретдинова Розалия · Суркова Арина · Каменева Мария · Клепикова Дарья</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>1:34.92</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>94.92</t>
         </is>
@@ -2463,12 +2465,12 @@
           <t>Каменева Мария · Годун Ника · Суркова Арина · Клепикова Дарья</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>1:44.19</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>104.19</t>
         </is>
@@ -2515,12 +2517,12 @@
           <t>Клепикова Дарья · Трофимова Дарья · Степанова Милана · Суркова Арина</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>3:28.73</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>208.73</t>
         </is>
@@ -2567,12 +2569,12 @@
           <t>Агапитова Елизавета · Чикунова Евгения · Суркова Арина · Клепикова Дарья</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>3:49.35</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>229.35</t>
         </is>
@@ -2619,12 +2621,12 @@
           <t>Егорова Анна · Муллакаева Дарья · Гуженкова Анастасия · Андрусенко Вероника</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>7:36.64</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>456.64</t>
         </is>
@@ -2667,12 +2669,12 @@
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>23.55</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>23.55</t>
         </is>
@@ -2715,12 +2717,12 @@
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>26.46</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>26.46</t>
         </is>
@@ -2763,12 +2765,12 @@
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>22.59</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>22.59</t>
         </is>
@@ -2811,12 +2813,12 @@
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>21.06</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>21.06</t>
         </is>
@@ -2859,12 +2861,12 @@
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>51.82</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>51.82</t>
         </is>
@@ -2907,12 +2909,12 @@
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>58.53</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>58.53</t>
         </is>
@@ -2955,12 +2957,12 @@
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>50.70</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>50.70</t>
         </is>
@@ -3003,12 +3005,12 @@
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>46.96</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>46.96</t>
         </is>
@@ -3051,12 +3053,12 @@
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>1:53.23</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>113.23</t>
         </is>
@@ -3099,12 +3101,12 @@
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>2:06.12</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>126.12</t>
         </is>
@@ -3147,12 +3149,12 @@
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>1:54.31</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>114.31</t>
         </is>
@@ -3195,12 +3197,12 @@
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>1:43.90</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>103.90</t>
         </is>
@@ -3243,12 +3245,12 @@
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>1:56.75</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>116.75</t>
         </is>
@@ -3291,12 +3293,12 @@
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>3:43.45</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G59" s="2" t="inlineStr">
         <is>
           <t>223.45</t>
         </is>
@@ -3339,12 +3341,12 @@
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>4:08.05</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>248.05</t>
         </is>
@@ -3387,12 +3389,12 @@
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>7:42.47</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>462.47</t>
         </is>
@@ -3435,12 +3437,12 @@
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>14:41.13</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>881.13</t>
         </is>
@@ -3487,12 +3489,12 @@
           <t>Лагунов Евгений · Гречин Андрей · Изотов Данила · Сухоруков Александр</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>3:09.52</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>189.52</t>
         </is>
@@ -3539,12 +3541,12 @@
           <t>Лифинцев Мирон · Пригода Кирилл · Минаков Андрей · Корнев Егор</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>3:26.93</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>206.93</t>
         </is>
@@ -3591,12 +3593,12 @@
           <t>Лобинцев Никита · Полищук Михаил · Изотов Данила · Сухоруков Александр</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>6:59.15</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>419.15</t>
         </is>
@@ -3639,12 +3641,12 @@
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>22.11</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>22.11</t>
         </is>
@@ -3687,12 +3689,12 @@
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>25.48</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>25.48</t>
         </is>
@@ -3735,12 +3737,12 @@
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>21.73</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>21.73</t>
         </is>
@@ -3783,12 +3785,12 @@
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>20.31</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>20.31</t>
         </is>
@@ -3831,12 +3833,12 @@
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>48.58</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>48.58</t>
         </is>
@@ -3879,12 +3881,12 @@
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>55.49</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>55.49</t>
         </is>
@@ -3927,12 +3929,12 @@
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>48.48</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>48.48</t>
         </is>
@@ -3975,12 +3977,12 @@
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>44.95</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>44.95</t>
         </is>
@@ -4023,12 +4025,12 @@
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr">
+      <c r="F74" s="2" t="inlineStr">
         <is>
           <t>50.26</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr">
         <is>
           <t>50.26</t>
         </is>
@@ -4071,12 +4073,12 @@
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr">
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>1:46.11</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr">
         <is>
           <t>106.11</t>
         </is>
@@ -4119,12 +4121,12 @@
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>2:00.16</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr">
         <is>
           <t>120.16</t>
         </is>
@@ -4167,12 +4169,12 @@
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
-      <c r="F77" t="inlineStr">
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>1:49.46</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr">
         <is>
           <t>109.46</t>
         </is>
@@ -4215,12 +4217,12 @@
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr">
+      <c r="F78" s="2" t="inlineStr">
         <is>
           <t>1:40.08</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr">
+      <c r="G78" s="2" t="inlineStr">
         <is>
           <t>100.08</t>
         </is>
@@ -4263,12 +4265,12 @@
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>1:52.13</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>112.13</t>
         </is>
@@ -4311,12 +4313,12 @@
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr">
+      <c r="F80" s="2" t="inlineStr">
         <is>
           <t>3:35.30</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr">
+      <c r="G80" s="2" t="inlineStr">
         <is>
           <t>215.30</t>
         </is>
@@ -4359,12 +4361,12 @@
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr">
+      <c r="F81" s="2" t="inlineStr">
         <is>
           <t>3:56.47</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
+      <c r="G81" s="2" t="inlineStr">
         <is>
           <t>236.47</t>
         </is>
@@ -4407,12 +4409,12 @@
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>7:32.36</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>452.36</t>
         </is>
@@ -4455,12 +4457,12 @@
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
-      <c r="F83" t="inlineStr">
+      <c r="F83" s="2" t="inlineStr">
         <is>
           <t>14:16.13</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
+      <c r="G83" s="2" t="inlineStr">
         <is>
           <t>856.13</t>
         </is>
@@ -4507,12 +4509,12 @@
           <t>Морозов Владимир · Седов Евгений · Кузьменко Иван · Рылов Евгений</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr">
         <is>
           <t>1:22.22</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G84" s="2" t="inlineStr">
         <is>
           <t>82.22</t>
         </is>
@@ -4559,12 +4561,12 @@
           <t>Колесников Климент · Пригода Кирилл · Попков Александр · Морозов Владимир</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr">
         <is>
           <t>1:30.44</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
+      <c r="G85" s="2" t="inlineStr">
         <is>
           <t>90.44</t>
         </is>
@@ -4611,12 +4613,12 @@
           <t>Гринев Владислав · Фесиков Сергей · Морозов Владимир · Колесников Климент</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>3:03.11</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G86" s="2" t="inlineStr">
         <is>
           <t>183.11</t>
         </is>
@@ -4663,12 +4665,12 @@
           <t>Лифинцев Мирон · Пригода Кирилл · Минаков Андрей · Корнев Егор</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>3:18.68</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
+      <c r="G87" s="2" t="inlineStr">
         <is>
           <t>198.68</t>
         </is>
@@ -4715,12 +4717,12 @@
           <t>Малютин Мартин · Вековищев Михаил · Гирев Иван · Красных Александр</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>6:46.84</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr">
+      <c r="G88" s="2" t="inlineStr">
         <is>
           <t>406.84</t>
         </is>
@@ -4767,12 +4769,12 @@
           <t>Морозов Владимир · Гринев Владислав · Суркова Арина · Каменева Мария</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F89" s="2" t="inlineStr">
         <is>
           <t>1:28.31</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
+      <c r="G89" s="2" t="inlineStr">
         <is>
           <t>88.31</t>
         </is>
@@ -4819,12 +4821,12 @@
           <t>Лифинцев Мирон · Пригода Кирилл · Суркова Арина · Трофимова Дарья</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="F90" s="2" t="inlineStr">
         <is>
           <t>1:35.36</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr">
+      <c r="G90" s="2" t="inlineStr">
         <is>
           <t>95.36</t>
         </is>
@@ -4871,12 +4873,12 @@
           <t>Корнев Егор · Гирев Иван · Трофимова Дарья · Клепикова Дарья</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>3:19.68</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr">
+      <c r="G91" s="2" t="inlineStr">
         <is>
           <t>199.68</t>
         </is>
@@ -4923,12 +4925,12 @@
           <t>Лифинцев Мирон · Пригода Кирилл · Клепикова Дарья · Трофимова Дарья</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
+      <c r="F92" s="2" t="inlineStr">
         <is>
           <t>3:37.97</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr">
+      <c r="G92" s="2" t="inlineStr">
         <is>
           <t>217.97</t>
         </is>

</xml_diff>

<commit_message>
data: update records 2026-07-19
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Все" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Женщины, бассейн 50 м" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Женщины, бассейн 25 м" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Мужчины, бассейн 50 м" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Мужчины, бассейн 25 м" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Смешанные эстафеты" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Женщины, бассейн 50 м" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Женщины, бассейн 25 м" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мужчины, бассейн 50 м" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мужчины, бассейн 25 м" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смешанные эстафеты" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Theme toggle: implement mandatory three-tap cycle (obsidian → titan → auto)
Skill audit against brand system found the toggle stuck at two states with
permanent manual override — no way back to auto once clicked, violating the
current brandbook rule (confirmed against the canonical reference in
fina-point, which already has this behavior).

- Cycle obsidian → titan → auto → obsidian; only manual choice persists,
  auto = no localStorage key
- Sun/Monitor/Moon icons show where the next click leads (per components.md)
- data-theme-mode on <html>, set both by inline anti-flash script and by app.js
- Instant switch: .theme-switching class + forced reflow suppresses the
  0.15s hover transitions during the flip, preventing a color-bleed cascade
- Cross-tab sync via storage event
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Женщины, бассейн 50 м" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Женщины, бассейн 25 м" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мужчины, бассейн 50 м" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мужчины, бассейн 25 м" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смешанные эстафеты" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Все" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Женщины, бассейн 50 м" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Женщины, бассейн 25 м" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Мужчины, бассейн 50 м" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Мужчины, бассейн 25 м" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Смешанные эстафеты" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Theme toggle: drop auto mode, manual choice only
Back to a plain two-state obsidian/titan toggle per explicit request — no
system-preference following, not even as an initial guess. Default is
always obsidian (brand's primary lik); manual choice always persists.

- Removed the auto tap and matchMedia entirely from static/app.js and the
  inline anti-flash script
- Single fixed theme-color meta tag (was two, conditioned on
  prefers-color-scheme) — no longer meaningful without system-following
- Kept the .theme-switching instant-switch guard and cross-tab storage
  sync — both are independent of how many states the toggle has
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Женщины, бассейн 50 м" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Женщины, бассейн 25 м" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мужчины, бассейн 50 м" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мужчины, бассейн 25 м" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смешанные эстафеты" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Все" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Женщины, бассейн 50 м" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Женщины, бассейн 25 м" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Мужчины, бассейн 50 м" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Мужчины, бассейн 25 м" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Смешанные эстафеты" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Header: group By Borozdov with the wordmark, keep it visible on mobile
- Wrap wordmark + signature in .brand so they sit adjacent instead of
  floating at the header midpoint via space-between
- Signature no longer hidden below 719px; scales down through two narrow
  breakpoints (icon-only download button below 560px, tighter spacing and
  smaller type below 380px) so it never gets ellipsis-clipped, verified
  down to 320px viewport width
</commit_message>
<xml_diff>
--- a/public/records.xlsx
+++ b/public/records.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Все" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Женщины, бассейн 50 м" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Женщины, бассейн 25 м" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мужчины, бассейн 50 м" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мужчины, бассейн 25 м" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Смешанные эстафеты" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Все" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Женщины, бассейн 50 м" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Женщины, бассейн 25 м" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Мужчины, бассейн 50 м" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Мужчины, бассейн 25 м" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Смешанные эстафеты" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>